<commit_message>
Alinear la invitación del Excel con el flujo del sitio
La hoja «Inicio» invitaba a agendar el diagnóstico de 30 minutos y
enlazaba a /contacto. Desde que el diagnóstico empieza por el test, eso
ofrecía justo el atajo que el nuevo flujo quiere evitar: quien abre el
Excel creía poder saltarse el test y pedir la reunión.

Ahora pide el reenvío del archivo completado y enlaza a un correo con el
asunto ya puesto. El Excel repite el mismo trato que el sitio, y lo
repite en el momento en que la persona termina de responder.

La hoja está protegida, así que la celda B27 se reescribió en el XML del
paquete en vez de abrir el archivo: editarlo con una librería de Excel
habría descartado el gráfico de la hoja «Resultado». Se verificó que las
20 entradas del paquete, el gráfico, la protección y las 89 fórmulas de
Test y Resultado siguen intactas.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/descargas/test-de-madurez-operativa-2026.xlsx
+++ b/public/descargas/test-de-madurez-operativa-2026.xlsx
@@ -2095,8 +2095,8 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="9" t="str">
-        <f aca="false">HYPERLINK("https://www.procesosclaros.cl/contacto","¿Prefieres revisarlo conmigo? Agenda el diagnóstico gratuito de 30 minutos →")</f>
-        <v>¿Prefieres revisarlo conmigo? Agenda el diagnóstico gratuito de 30 minutos →</v>
+        <f aca="false">HYPERLINK("mailto:jorge@procesosclaros.cl?subject=Resultado%20del%20test%20de%20madurez","¿Quieres revisarlo conmigo? Envíame este archivo completado a jorge@procesosclaros.cl →")</f>
+        <v>¿Quieres revisarlo conmigo? Envíame este archivo completado a jorge@procesosclaros.cl →</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>